<commit_message>
agregar datos a la tabla
</commit_message>
<xml_diff>
--- a/gastos-personales.xlsx
+++ b/gastos-personales.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PERSONAL\Documents\CAMPUSLAND\CURSO-WEB-CAMPUS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9786E7E3-2F07-4CF5-BA7C-F0AE276BFAED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC018FA1-5803-400F-A7FA-C440CB54161D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A0B42D86-ABC7-4FEE-9329-62E168F97D9F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>GASTOS PERSONALES</t>
   </si>
@@ -51,6 +51,18 @@
   </si>
   <si>
     <t>GASTOS</t>
+  </si>
+  <si>
+    <t>arriendo</t>
+  </si>
+  <si>
+    <t>nomina</t>
+  </si>
+  <si>
+    <t>servicios</t>
+  </si>
+  <si>
+    <t>alimentacion</t>
   </si>
 </sst>
 </file>
@@ -101,14 +113,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -443,23 +454,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E773FCF-72EA-4356-AA0E-FEC31F16AB6F}">
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -472,165 +478,114 @@
       <c r="D2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="3">
+        <v>46296</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="1">
+        <v>2000000</v>
+      </c>
       <c r="D3" s="1"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="3">
+        <v>46296</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>5</v>
+      </c>
       <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
+      <c r="D4" s="1">
+        <v>500000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="3">
+        <v>46296</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>7</v>
+      </c>
       <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
+      <c r="D5" s="1">
+        <v>200000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="3">
+        <v>46296</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>8</v>
+      </c>
       <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D6" s="1">
+        <v>600000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="3"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-      <c r="I10" s="3"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
-      <c r="I11" s="3"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-      <c r="I15" s="3"/>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="3"/>
-      <c r="G16" s="3"/>
-      <c r="H16" s="3"/>
-      <c r="I16" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>